<commit_message>
Local edits before pulling remote
</commit_message>
<xml_diff>
--- a/data/forest_plots.xlsx
+++ b/data/forest_plots.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rkuo/Documents/DPhil/Umbrella review/Submission folder/bmj/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rkuo/Documents/DPhil/Umbrella review/umbrella_test/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B41B76A-42B2-414A-A755-4D3DE26F7328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBB82DE3-A6DF-CC4A-808C-D4FB7425D104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36800" yWindow="2120" windowWidth="27240" windowHeight="16440" activeTab="2" xr2:uid="{2D65041E-0903-544A-A28B-F087D47BCED9}"/>
+    <workbookView xWindow="540" yWindow="1220" windowWidth="27240" windowHeight="16440" activeTab="2" xr2:uid="{2D65041E-0903-544A-A28B-F087D47BCED9}"/>
   </bookViews>
   <sheets>
     <sheet name="All" sheetId="1" r:id="rId1"/>
     <sheet name="Comparators" sheetId="2" r:id="rId2"/>
     <sheet name="Subgroups" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -264,11 +264,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -667,7 +666,7 @@
       <c r="F2">
         <v>0.91100000000000003</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2">
         <v>7.9000000000000001E-2</v>
       </c>
       <c r="H2">
@@ -685,7 +684,7 @@
       <c r="L2">
         <v>0.91600000000000004</v>
       </c>
-      <c r="M2" s="3">
+      <c r="M2">
         <v>7.0999999999999994E-2</v>
       </c>
       <c r="N2">
@@ -1605,7 +1604,7 @@
       <c r="F2">
         <v>0.91100000000000003</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2">
         <v>7.9000000000000001E-2</v>
       </c>
       <c r="H2">
@@ -1623,7 +1622,7 @@
       <c r="L2">
         <v>0.91600000000000004</v>
       </c>
-      <c r="M2" s="3">
+      <c r="M2">
         <v>7.0999999999999994E-2</v>
       </c>
       <c r="N2">
@@ -1698,7 +1697,7 @@
         <v>93.2</v>
       </c>
       <c r="R3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S3" t="s">
         <v>19</v>
@@ -2543,7 +2542,7 @@
       <c r="F18">
         <v>0.91100000000000003</v>
       </c>
-      <c r="G18" s="3">
+      <c r="G18">
         <v>7.9000000000000001E-2</v>
       </c>
       <c r="H18">
@@ -2561,7 +2560,7 @@
       <c r="L18">
         <v>0.91600000000000004</v>
       </c>
-      <c r="M18" s="3">
+      <c r="M18">
         <v>7.0999999999999994E-2</v>
       </c>
       <c r="N18">

</xml_diff>